<commit_message>
Record source md5 and build in Protocol sheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T6gEewJ8YaCdmnsfS34RJd
</commit_message>
<xml_diff>
--- a/results/final_results.xlsx
+++ b/results/final_results.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -511,6 +511,54 @@
       <c r="B7" t="inlineStr">
         <is>
           <t>double (seq and par byte-identical, same LBG iteration count)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>sem_v3.c md5</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>02e8379fe098ced39515ab51941c3872</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>pam_v4.c md5</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>f1b1687d85bbf734541c264cb11f24c6</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>gcc -O2 -Wall -Wextra ... -lm ; mpicc -O2 -Wall -Wextra ... -lm</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Campaign</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>run_timing_12.sh, NPS=2 4 6 8 10 12 14, single session; checks md5 verified before the run</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Chapter 4 review and replacement tables; correct overstated 9.3x 'theoretical limit' wording
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T6gEewJ8YaCdmnsfS34RJd
</commit_message>
<xml_diff>
--- a/results/final_results.xlsx
+++ b/results/final_results.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Speedup LBG" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Speedup Total" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Efficiency %" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ch4 tables (replace 4.4-4.8)" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6307,4 +6308,770 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Table 4.4/4.5 replacement: sequential times (s) and iterations</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>LBG_s</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Total_s</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>iters</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>LBG ms/iter</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.2639</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.3483</v>
+      </c>
+      <c r="D3" t="n">
+        <v>160</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1.649</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>boat_img</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.2322</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.3169</v>
+      </c>
+      <c r="D4" t="n">
+        <v>151</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1.538</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>cameraman_img</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.2374</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.3226</v>
+      </c>
+      <c r="D5" t="n">
+        <v>155</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1.532</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>peppers_img</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.2808</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.3651</v>
+      </c>
+      <c r="D6" t="n">
+        <v>132</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2.127</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>chest_xray2_img</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.2331</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.3175</v>
+      </c>
+      <c r="D7" t="n">
+        <v>125</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1.865</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>mammo2_img</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.2086</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.2922</v>
+      </c>
+      <c r="D8" t="n">
+        <v>98</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2.129</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>lung_ct2_img</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.2909</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.376</v>
+      </c>
+      <c r="D9" t="n">
+        <v>197</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1.477</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>brain_mri2_img</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.2452</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.3281</v>
+      </c>
+      <c r="D10" t="n">
+        <v>142</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1.727</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>lena_color</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.7677</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.9741</v>
+      </c>
+      <c r="D11" t="n">
+        <v>476</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1.613</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>retina2_color</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.6573</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.864</v>
+      </c>
+      <c r="D12" t="n">
+        <v>493</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1.333</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>brain_pet3_color</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.805</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1.0114</v>
+      </c>
+      <c r="D13" t="n">
+        <v>495</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1.626</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>brain_pet4_color</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.7811</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.9869</v>
+      </c>
+      <c r="D14" t="n">
+        <v>502</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1.556</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>Table 4.6 replacement: LBG speedup, mean over 12 images</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="n"/>
+      <c r="C16" s="1" t="n"/>
+      <c r="D16" s="1" t="n"/>
+      <c r="E16" s="1" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>np</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>mean speedup</t>
+        </is>
+      </c>
+      <c r="C17" s="1" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="D17" s="1" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="E17" s="1" t="inlineStr">
+        <is>
+          <t>efficiency %</t>
+        </is>
+      </c>
+      <c r="F17" s="1" t="inlineStr">
+        <is>
+          <t>Karp-Flatt e</t>
+        </is>
+      </c>
+      <c r="G17" s="1" t="inlineStr">
+        <is>
+          <t>capacity-weighted ideal</t>
+        </is>
+      </c>
+      <c r="H17" s="1" t="inlineStr">
+        <is>
+          <t>fraction of ideal</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>2</v>
+      </c>
+      <c r="B18" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="C18" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="E18" t="n">
+        <v>96</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.0417</v>
+      </c>
+      <c r="G18" t="n">
+        <v>2</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.96</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>4</v>
+      </c>
+      <c r="B19" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="C19" t="n">
+        <v>3.73</v>
+      </c>
+      <c r="D19" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="E19" t="n">
+        <v>94</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.0214</v>
+      </c>
+      <c r="G19" t="n">
+        <v>4</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>6</v>
+      </c>
+      <c r="B20" t="n">
+        <v>5.37</v>
+      </c>
+      <c r="C20" t="n">
+        <v>5.34</v>
+      </c>
+      <c r="D20" t="n">
+        <v>5.39</v>
+      </c>
+      <c r="E20" t="n">
+        <v>89.40000000000001</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.0236</v>
+      </c>
+      <c r="G20" t="n">
+        <v>6</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.894</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>8</v>
+      </c>
+      <c r="B21" t="n">
+        <v>6.27</v>
+      </c>
+      <c r="C21" t="n">
+        <v>6.24</v>
+      </c>
+      <c r="D21" t="n">
+        <v>6.31</v>
+      </c>
+      <c r="E21" t="n">
+        <v>78.40000000000001</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.0393</v>
+      </c>
+      <c r="G21" t="n">
+        <v>7.28</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.861</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>10</v>
+      </c>
+      <c r="B22" t="n">
+        <v>7.31</v>
+      </c>
+      <c r="C22" t="n">
+        <v>7.28</v>
+      </c>
+      <c r="D22" t="n">
+        <v>7.34</v>
+      </c>
+      <c r="E22" t="n">
+        <v>73.09999999999999</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.0408</v>
+      </c>
+      <c r="G22" t="n">
+        <v>8.57</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0.854</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>12</v>
+      </c>
+      <c r="B23" t="n">
+        <v>8.18</v>
+      </c>
+      <c r="C23" t="n">
+        <v>8.140000000000001</v>
+      </c>
+      <c r="D23" t="n">
+        <v>8.210000000000001</v>
+      </c>
+      <c r="E23" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.0425</v>
+      </c>
+      <c r="G23" t="n">
+        <v>9.85</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.83</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>14</v>
+      </c>
+      <c r="B24" t="n">
+        <v>9.119999999999999</v>
+      </c>
+      <c r="C24" t="n">
+        <v>9.029999999999999</v>
+      </c>
+      <c r="D24" t="n">
+        <v>9.18</v>
+      </c>
+      <c r="E24" t="n">
+        <v>65.09999999999999</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.0412</v>
+      </c>
+      <c r="G24" t="n">
+        <v>11.13</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0.819</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>Table 4.8 replacement: Total speedup, mean over 12 images (gray 8, color 4)</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="n"/>
+      <c r="C26" s="1" t="n"/>
+      <c r="D26" s="1" t="n"/>
+      <c r="E26" s="1" t="n"/>
+      <c r="F26" s="1" t="n"/>
+      <c r="G26" s="1" t="n"/>
+      <c r="H26" s="1" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>np</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="inlineStr">
+        <is>
+          <t>mean all</t>
+        </is>
+      </c>
+      <c r="C27" s="1" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="D27" s="1" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="E27" s="1" t="inlineStr">
+        <is>
+          <t>efficiency %</t>
+        </is>
+      </c>
+      <c r="F27" s="1" t="inlineStr">
+        <is>
+          <t>Karp-Flatt e</t>
+        </is>
+      </c>
+      <c r="G27" s="1" t="inlineStr">
+        <is>
+          <t>mean gray</t>
+        </is>
+      </c>
+      <c r="H27" s="1" t="inlineStr">
+        <is>
+          <t>mean color</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>2</v>
+      </c>
+      <c r="B28" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="C28" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="D28" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="E28" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.1423</v>
+      </c>
+      <c r="G28" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="H28" t="n">
+        <v>1.81</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>4</v>
+      </c>
+      <c r="B29" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="C29" t="n">
+        <v>2.73</v>
+      </c>
+      <c r="D29" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="E29" t="n">
+        <v>73.7</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0.1189</v>
+      </c>
+      <c r="G29" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="H29" t="n">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>6</v>
+      </c>
+      <c r="B30" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="C30" t="n">
+        <v>3.36</v>
+      </c>
+      <c r="D30" t="n">
+        <v>4.21</v>
+      </c>
+      <c r="E30" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.1235</v>
+      </c>
+      <c r="G30" t="n">
+        <v>3.48</v>
+      </c>
+      <c r="H30" t="n">
+        <v>4.16</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>8</v>
+      </c>
+      <c r="B31" t="n">
+        <v>3.94</v>
+      </c>
+      <c r="C31" t="n">
+        <v>3.48</v>
+      </c>
+      <c r="D31" t="n">
+        <v>4.54</v>
+      </c>
+      <c r="E31" t="n">
+        <v>49.2</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0.1473</v>
+      </c>
+      <c r="G31" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="H31" t="n">
+        <v>4.47</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>10</v>
+      </c>
+      <c r="B32" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="C32" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="D32" t="n">
+        <v>5.08</v>
+      </c>
+      <c r="E32" t="n">
+        <v>43.3</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.1454</v>
+      </c>
+      <c r="G32" t="n">
+        <v>4</v>
+      </c>
+      <c r="H32" t="n">
+        <v>4.99</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>12</v>
+      </c>
+      <c r="B33" t="n">
+        <v>4.62</v>
+      </c>
+      <c r="C33" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="D33" t="n">
+        <v>5.47</v>
+      </c>
+      <c r="E33" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0.1453</v>
+      </c>
+      <c r="G33" t="n">
+        <v>4.23</v>
+      </c>
+      <c r="H33" t="n">
+        <v>5.4</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>14</v>
+      </c>
+      <c r="B34" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="C34" t="n">
+        <v>4.17</v>
+      </c>
+      <c r="D34" t="n">
+        <v>5.91</v>
+      </c>
+      <c r="E34" t="n">
+        <v>35</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.143</v>
+      </c>
+      <c r="G34" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="H34" t="n">
+        <v>5.79</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Note: capacity-weighted ideal uses P=275, E=176.5 Mcmp/s (ratio 0.642) from the calibration benchmark; it is a model, not a measurement.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Equal vs Adaptive results (v4, 12 images), model check, IMGS override in run_eq_ad.sh
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T6gEewJ8YaCdmnsfS34RJd
</commit_message>
<xml_diff>
--- a/results/final_results.xlsx
+++ b/results/final_results.xlsx
@@ -15,6 +15,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Speedup Total" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Efficiency %" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ch4 tables (replace 4.4-4.8)" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equal vs Adaptive" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EqAd summary" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -568,6 +570,234 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>np</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>mean gain %</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>images where Adaptive faster</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>mean gain % (without retina)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>model-predicted gain %</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B2" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B3" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="C3" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="D3" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="C4" t="n">
+        <v>-1.3</v>
+      </c>
+      <c r="D4" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B5" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="C5" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="D5" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="E5" t="n">
+        <v>12</v>
+      </c>
+      <c r="F5" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="G5" t="n">
+        <v>29.5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B6" t="n">
+        <v>23.7</v>
+      </c>
+      <c r="C6" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="E6" t="n">
+        <v>12</v>
+      </c>
+      <c r="F6" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>25.1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>12</v>
+      </c>
+      <c r="B7" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="C7" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="D7" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="E7" t="n">
+        <v>12</v>
+      </c>
+      <c r="F7" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="G7" t="n">
+        <v>21.8</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>14</v>
+      </c>
+      <c r="B8" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="C8" t="n">
+        <v>15</v>
+      </c>
+      <c r="D8" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="E8" t="n">
+        <v>12</v>
+      </c>
+      <c r="F8" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="G8" t="n">
+        <v>19.3</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Model: gain = 1 - np*r/(6+(np-6)*r), r = E/P speed = 176.5/275 = 0.642. Retina np=4..10 rows are suspected disturbed runs; rerun pending.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -7074,4 +7304,2180 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G85"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>mode</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>np</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>equal_s</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>adaptive_s</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>adaptive_gain_pct</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>flag</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.1375</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.1375</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.0698</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.0698</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>6</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.0492</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.0492</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.0589</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.0421</v>
+      </c>
+      <c r="F5" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.0476</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.0361</v>
+      </c>
+      <c r="F6" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="G6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>12</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.0406</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.0322</v>
+      </c>
+      <c r="F7" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="G7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>14</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.0352</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.0288</v>
+      </c>
+      <c r="F8" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="G8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>boat_img</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.1209</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.1207</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>boat_img</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.061</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.0615</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>boat_img</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>6</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.0431</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.0436</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-1.2</v>
+      </c>
+      <c r="G11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>boat_img</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>8</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.0517</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.0371</v>
+      </c>
+      <c r="F12" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="G12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>boat_img</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>10</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.0417</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.0318</v>
+      </c>
+      <c r="F13" t="n">
+        <v>23.7</v>
+      </c>
+      <c r="G13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>boat_img</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>12</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.0358</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.0284</v>
+      </c>
+      <c r="F14" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="G14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>boat_img</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>14</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.031</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.0255</v>
+      </c>
+      <c r="F15" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="G15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>cameraman_img</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.1232</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.1235</v>
+      </c>
+      <c r="F16" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="G16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>cameraman_img</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>4</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.06270000000000001</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.0624</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>cameraman_img</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>6</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.044</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.044</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>cameraman_img</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>8</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.0528</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.0377</v>
+      </c>
+      <c r="F19" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="G19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>cameraman_img</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>10</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.0428</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.0325</v>
+      </c>
+      <c r="F20" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="G20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>cameraman_img</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>12</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.0366</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.0292</v>
+      </c>
+      <c r="F21" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="G21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>cameraman_img</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>14</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0.0317</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="F22" t="n">
+        <v>18</v>
+      </c>
+      <c r="G22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>peppers_img</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0.1459</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0.1458</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>peppers_img</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>4</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0.0737</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.074</v>
+      </c>
+      <c r="F24" t="n">
+        <v>-0.4</v>
+      </c>
+      <c r="G24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>peppers_img</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>6</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0.052</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.0521</v>
+      </c>
+      <c r="F25" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="G25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>peppers_img</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>8</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0.0626</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.0446</v>
+      </c>
+      <c r="F26" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="G26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>peppers_img</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>10</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.0504</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.0381</v>
+      </c>
+      <c r="F27" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="G27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>peppers_img</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>12</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0.043</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="F28" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="G28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>peppers_img</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>14</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0.0372</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.0305</v>
+      </c>
+      <c r="F29" t="n">
+        <v>18</v>
+      </c>
+      <c r="G29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>chest_xray2_img</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>2</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0.1209</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0.1211</v>
+      </c>
+      <c r="F30" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="G30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>chest_xray2_img</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>4</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0.0615</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0.0614</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>chest_xray2_img</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>6</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0.0432</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="F32" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="G32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>chest_xray2_img</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>8</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0.052</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0.0372</v>
+      </c>
+      <c r="F33" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="G33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>chest_xray2_img</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>10</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0.0419</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0.0319</v>
+      </c>
+      <c r="F34" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="G34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>chest_xray2_img</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>12</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0.036</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0.0286</v>
+      </c>
+      <c r="F35" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="G35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>chest_xray2_img</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>14</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0.0312</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0.0256</v>
+      </c>
+      <c r="F36" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="G36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>mammo2_img</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>2</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0.1084</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0.1086</v>
+      </c>
+      <c r="F37" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="G37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>mammo2_img</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>4</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0.0548</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0.0548</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>mammo2_img</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>6</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0.0388</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0.0388</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>mammo2_img</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>8</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0.0465</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0.0331</v>
+      </c>
+      <c r="F40" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="G40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>mammo2_img</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>10</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0.0375</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0.0284</v>
+      </c>
+      <c r="F41" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="G41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>mammo2_img</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>12</v>
+      </c>
+      <c r="D42" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0.0254</v>
+      </c>
+      <c r="F42" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="G42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>mammo2_img</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>14</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0.0277</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0.0227</v>
+      </c>
+      <c r="F43" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="G43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>lung_ct2_img</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>2</v>
+      </c>
+      <c r="D44" t="n">
+        <v>0.1514</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0.1516</v>
+      </c>
+      <c r="F44" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="G44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>lung_ct2_img</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>4</v>
+      </c>
+      <c r="D45" t="n">
+        <v>0.0766</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0.0769</v>
+      </c>
+      <c r="F45" t="n">
+        <v>-0.4</v>
+      </c>
+      <c r="G45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>lung_ct2_img</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>6</v>
+      </c>
+      <c r="D46" t="n">
+        <v>0.0544</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0.0551</v>
+      </c>
+      <c r="F46" t="n">
+        <v>-1.3</v>
+      </c>
+      <c r="G46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>lung_ct2_img</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>8</v>
+      </c>
+      <c r="D47" t="n">
+        <v>0.0646</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0.0463</v>
+      </c>
+      <c r="F47" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="G47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>lung_ct2_img</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>10</v>
+      </c>
+      <c r="D48" t="n">
+        <v>0.0523</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0.0398</v>
+      </c>
+      <c r="F48" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="G48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>lung_ct2_img</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>12</v>
+      </c>
+      <c r="D49" t="n">
+        <v>0.0446</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0.0354</v>
+      </c>
+      <c r="F49" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="G49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>lung_ct2_img</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>14</v>
+      </c>
+      <c r="D50" t="n">
+        <v>0.0387</v>
+      </c>
+      <c r="E50" t="n">
+        <v>0.0317</v>
+      </c>
+      <c r="F50" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="G50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>brain_mri2_img</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>2</v>
+      </c>
+      <c r="D51" t="n">
+        <v>0.1276</v>
+      </c>
+      <c r="E51" t="n">
+        <v>0.1282</v>
+      </c>
+      <c r="F51" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="G51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>brain_mri2_img</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>4</v>
+      </c>
+      <c r="D52" t="n">
+        <v>0.0643</v>
+      </c>
+      <c r="E52" t="n">
+        <v>0.06469999999999999</v>
+      </c>
+      <c r="F52" t="n">
+        <v>-0.6</v>
+      </c>
+      <c r="G52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>brain_mri2_img</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>6</v>
+      </c>
+      <c r="D53" t="n">
+        <v>0.0457</v>
+      </c>
+      <c r="E53" t="n">
+        <v>0.0457</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>brain_mri2_img</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>8</v>
+      </c>
+      <c r="D54" t="n">
+        <v>0.0545</v>
+      </c>
+      <c r="E54" t="n">
+        <v>0.039</v>
+      </c>
+      <c r="F54" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="G54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>brain_mri2_img</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>10</v>
+      </c>
+      <c r="D55" t="n">
+        <v>0.044</v>
+      </c>
+      <c r="E55" t="n">
+        <v>0.0333</v>
+      </c>
+      <c r="F55" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="G55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>brain_mri2_img</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>12</v>
+      </c>
+      <c r="D56" t="n">
+        <v>0.0376</v>
+      </c>
+      <c r="E56" t="n">
+        <v>0.0298</v>
+      </c>
+      <c r="F56" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="G56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>brain_mri2_img</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>14</v>
+      </c>
+      <c r="D57" t="n">
+        <v>0.0325</v>
+      </c>
+      <c r="E57" t="n">
+        <v>0.0267</v>
+      </c>
+      <c r="F57" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="G57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>lena_color</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>2</v>
+      </c>
+      <c r="D58" t="n">
+        <v>0.4001</v>
+      </c>
+      <c r="E58" t="n">
+        <v>0.4003</v>
+      </c>
+      <c r="F58" t="n">
+        <v>-0</v>
+      </c>
+      <c r="G58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>lena_color</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>4</v>
+      </c>
+      <c r="D59" t="n">
+        <v>0.2023</v>
+      </c>
+      <c r="E59" t="n">
+        <v>0.2031</v>
+      </c>
+      <c r="F59" t="n">
+        <v>-0.4</v>
+      </c>
+      <c r="G59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>lena_color</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>6</v>
+      </c>
+      <c r="D60" t="n">
+        <v>0.1433</v>
+      </c>
+      <c r="E60" t="n">
+        <v>0.1433</v>
+      </c>
+      <c r="F60" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>lena_color</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>8</v>
+      </c>
+      <c r="D61" t="n">
+        <v>0.1714</v>
+      </c>
+      <c r="E61" t="n">
+        <v>0.1221</v>
+      </c>
+      <c r="F61" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="G61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>lena_color</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>10</v>
+      </c>
+      <c r="D62" t="n">
+        <v>0.1378</v>
+      </c>
+      <c r="E62" t="n">
+        <v>0.1048</v>
+      </c>
+      <c r="F62" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="G62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>lena_color</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>12</v>
+      </c>
+      <c r="D63" t="n">
+        <v>0.1176</v>
+      </c>
+      <c r="E63" t="n">
+        <v>0.0934</v>
+      </c>
+      <c r="F63" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="G63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>lena_color</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>14</v>
+      </c>
+      <c r="D64" t="n">
+        <v>0.1018</v>
+      </c>
+      <c r="E64" t="n">
+        <v>0.08649999999999999</v>
+      </c>
+      <c r="F64" t="n">
+        <v>15</v>
+      </c>
+      <c r="G64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>retina2_color</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>2</v>
+      </c>
+      <c r="D65" t="n">
+        <v>0.3416</v>
+      </c>
+      <c r="E65" t="n">
+        <v>0.342</v>
+      </c>
+      <c r="F65" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="G65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>retina2_color</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>4</v>
+      </c>
+      <c r="D66" t="n">
+        <v>0.2438</v>
+      </c>
+      <c r="E66" t="n">
+        <v>0.1919</v>
+      </c>
+      <c r="F66" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>rerun pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>retina2_color</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>6</v>
+      </c>
+      <c r="D67" t="n">
+        <v>0.1683</v>
+      </c>
+      <c r="E67" t="n">
+        <v>0.1387</v>
+      </c>
+      <c r="F67" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>rerun pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>retina2_color</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>8</v>
+      </c>
+      <c r="D68" t="n">
+        <v>0.1473</v>
+      </c>
+      <c r="E68" t="n">
+        <v>0.1095</v>
+      </c>
+      <c r="F68" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>rerun pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>retina2_color</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>10</v>
+      </c>
+      <c r="D69" t="n">
+        <v>0.1186</v>
+      </c>
+      <c r="E69" t="n">
+        <v>0.0959</v>
+      </c>
+      <c r="F69" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>rerun pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>retina2_color</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>12</v>
+      </c>
+      <c r="D70" t="n">
+        <v>0.101</v>
+      </c>
+      <c r="E70" t="n">
+        <v>0.0804</v>
+      </c>
+      <c r="F70" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="G70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>retina2_color</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>14</v>
+      </c>
+      <c r="D71" t="n">
+        <v>0.0873</v>
+      </c>
+      <c r="E71" t="n">
+        <v>0.0716</v>
+      </c>
+      <c r="F71" t="n">
+        <v>18</v>
+      </c>
+      <c r="G71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>brain_pet3_color</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>2</v>
+      </c>
+      <c r="D72" t="n">
+        <v>0.4175</v>
+      </c>
+      <c r="E72" t="n">
+        <v>0.4187</v>
+      </c>
+      <c r="F72" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="G72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>brain_pet3_color</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>4</v>
+      </c>
+      <c r="D73" t="n">
+        <v>0.2116</v>
+      </c>
+      <c r="E73" t="n">
+        <v>0.213</v>
+      </c>
+      <c r="F73" t="n">
+        <v>-0.7</v>
+      </c>
+      <c r="G73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>brain_pet3_color</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>6</v>
+      </c>
+      <c r="D74" t="n">
+        <v>0.149</v>
+      </c>
+      <c r="E74" t="n">
+        <v>0.1493</v>
+      </c>
+      <c r="F74" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="G74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>brain_pet3_color</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>8</v>
+      </c>
+      <c r="D75" t="n">
+        <v>0.1798</v>
+      </c>
+      <c r="E75" t="n">
+        <v>0.1284</v>
+      </c>
+      <c r="F75" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="G75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>brain_pet3_color</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>10</v>
+      </c>
+      <c r="D76" t="n">
+        <v>0.1452</v>
+      </c>
+      <c r="E76" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="F76" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="G76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>brain_pet3_color</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>12</v>
+      </c>
+      <c r="D77" t="n">
+        <v>0.1237</v>
+      </c>
+      <c r="E77" t="n">
+        <v>0.0984</v>
+      </c>
+      <c r="F77" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="G77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>brain_pet3_color</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>14</v>
+      </c>
+      <c r="D78" t="n">
+        <v>0.1069</v>
+      </c>
+      <c r="E78" t="n">
+        <v>0.0877</v>
+      </c>
+      <c r="F78" t="n">
+        <v>18</v>
+      </c>
+      <c r="G78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>brain_pet4_color</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>2</v>
+      </c>
+      <c r="D79" t="n">
+        <v>0.4073</v>
+      </c>
+      <c r="E79" t="n">
+        <v>0.4092</v>
+      </c>
+      <c r="F79" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="G79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>brain_pet4_color</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>4</v>
+      </c>
+      <c r="D80" t="n">
+        <v>0.2064</v>
+      </c>
+      <c r="E80" t="n">
+        <v>0.2063</v>
+      </c>
+      <c r="F80" t="n">
+        <v>0</v>
+      </c>
+      <c r="G80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>brain_pet4_color</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>6</v>
+      </c>
+      <c r="D81" t="n">
+        <v>0.1455</v>
+      </c>
+      <c r="E81" t="n">
+        <v>0.1454</v>
+      </c>
+      <c r="F81" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>brain_pet4_color</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>8</v>
+      </c>
+      <c r="D82" t="n">
+        <v>0.1743</v>
+      </c>
+      <c r="E82" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="F82" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="G82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>brain_pet4_color</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>10</v>
+      </c>
+      <c r="D83" t="n">
+        <v>0.1405</v>
+      </c>
+      <c r="E83" t="n">
+        <v>0.1065</v>
+      </c>
+      <c r="F83" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="G83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>brain_pet4_color</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>12</v>
+      </c>
+      <c r="D84" t="n">
+        <v>0.1197</v>
+      </c>
+      <c r="E84" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="F84" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="G84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>brain_pet4_color</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>14</v>
+      </c>
+      <c r="D85" t="n">
+        <v>0.1035</v>
+      </c>
+      <c r="E85" t="n">
+        <v>0.0849</v>
+      </c>
+      <c r="F85" t="n">
+        <v>18</v>
+      </c>
+      <c r="G85" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Replace Retina Equal/Adaptive rows with rerun; finalize summary
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T6gEewJ8YaCdmnsfS34RJd
</commit_message>
<xml_diff>
--- a/results/final_results.xlsx
+++ b/results/final_results.xlsx
@@ -576,16 +576,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -611,15 +610,10 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>images where Adaptive faster</t>
+          <t>images where Adaptive faster (&gt;0.5%)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>mean gain % (without retina)</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>model-predicted gain %</t>
         </is>
@@ -630,7 +624,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>-0.1</v>
+        <v>-0.2</v>
       </c>
       <c r="C2" t="n">
         <v>-0.5</v>
@@ -642,9 +636,6 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.2</v>
-      </c>
-      <c r="G2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -653,21 +644,18 @@
         <v>4</v>
       </c>
       <c r="B3" t="n">
-        <v>1.6</v>
+        <v>-0.2</v>
       </c>
       <c r="C3" t="n">
         <v>-0.8</v>
       </c>
       <c r="D3" t="n">
-        <v>21.3</v>
+        <v>0.5</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.2</v>
-      </c>
-      <c r="G3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -676,21 +664,18 @@
         <v>6</v>
       </c>
       <c r="B4" t="n">
-        <v>1.2</v>
+        <v>-0.3</v>
       </c>
       <c r="C4" t="n">
         <v>-1.3</v>
       </c>
       <c r="D4" t="n">
-        <v>17.6</v>
+        <v>0.1</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.3</v>
-      </c>
-      <c r="G4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -699,10 +684,10 @@
         <v>8</v>
       </c>
       <c r="B5" t="n">
-        <v>28.3</v>
+        <v>28.5</v>
       </c>
       <c r="C5" t="n">
-        <v>25.7</v>
+        <v>28.2</v>
       </c>
       <c r="D5" t="n">
         <v>28.8</v>
@@ -711,9 +696,6 @@
         <v>12</v>
       </c>
       <c r="F5" t="n">
-        <v>28.5</v>
-      </c>
-      <c r="G5" t="n">
         <v>29.5</v>
       </c>
     </row>
@@ -722,10 +704,10 @@
         <v>10</v>
       </c>
       <c r="B6" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="C6" t="n">
         <v>23.7</v>
-      </c>
-      <c r="C6" t="n">
-        <v>19.1</v>
       </c>
       <c r="D6" t="n">
         <v>24.4</v>
@@ -734,9 +716,6 @@
         <v>12</v>
       </c>
       <c r="F6" t="n">
-        <v>24.1</v>
-      </c>
-      <c r="G6" t="n">
         <v>25.1</v>
       </c>
     </row>
@@ -757,9 +736,6 @@
         <v>12</v>
       </c>
       <c r="F7" t="n">
-        <v>20.6</v>
-      </c>
-      <c r="G7" t="n">
         <v>21.8</v>
       </c>
     </row>
@@ -780,16 +756,13 @@
         <v>12</v>
       </c>
       <c r="F8" t="n">
-        <v>17.7</v>
-      </c>
-      <c r="G8" t="n">
         <v>19.3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Model: gain = 1 - np*r/(6+(np-6)*r), r = E/P speed = 176.5/275 = 0.642. Retina np=4..10 rows are suspected disturbed runs; rerun pending.</t>
+          <t>Model: gain = 1 - np*r/(6+(np-6)*r), r = E/P speed = 176.5/275 = 0.642. Retina rows replaced by a rerun (eq_ad_retina.csv).</t>
         </is>
       </c>
     </row>
@@ -7312,16 +7285,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G85"/>
+  <dimension ref="A1:F85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7355,11 +7327,6 @@
           <t>adaptive_gain_pct</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>flag</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -7384,7 +7351,6 @@
       <c r="F2" t="n">
         <v>0</v>
       </c>
-      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -7409,7 +7375,6 @@
       <c r="F3" t="n">
         <v>0</v>
       </c>
-      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -7434,7 +7399,6 @@
       <c r="F4" t="n">
         <v>0</v>
       </c>
-      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -7459,7 +7423,6 @@
       <c r="F5" t="n">
         <v>28.5</v>
       </c>
-      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -7484,7 +7447,6 @@
       <c r="F6" t="n">
         <v>24.2</v>
       </c>
-      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -7509,7 +7471,6 @@
       <c r="F7" t="n">
         <v>20.7</v>
       </c>
-      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -7534,7 +7495,6 @@
       <c r="F8" t="n">
         <v>18.2</v>
       </c>
-      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -7559,7 +7519,6 @@
       <c r="F9" t="n">
         <v>0.2</v>
       </c>
-      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -7584,7 +7543,6 @@
       <c r="F10" t="n">
         <v>-0.8</v>
       </c>
-      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -7609,7 +7567,6 @@
       <c r="F11" t="n">
         <v>-1.2</v>
       </c>
-      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -7634,7 +7591,6 @@
       <c r="F12" t="n">
         <v>28.2</v>
       </c>
-      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -7659,7 +7615,6 @@
       <c r="F13" t="n">
         <v>23.7</v>
       </c>
-      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -7684,7 +7639,6 @@
       <c r="F14" t="n">
         <v>20.7</v>
       </c>
-      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -7709,7 +7663,6 @@
       <c r="F15" t="n">
         <v>17.7</v>
       </c>
-      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -7734,7 +7687,6 @@
       <c r="F16" t="n">
         <v>-0.2</v>
       </c>
-      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -7759,7 +7711,6 @@
       <c r="F17" t="n">
         <v>0.5</v>
       </c>
-      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -7784,7 +7735,6 @@
       <c r="F18" t="n">
         <v>0</v>
       </c>
-      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -7809,7 +7759,6 @@
       <c r="F19" t="n">
         <v>28.6</v>
       </c>
-      <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -7834,7 +7783,6 @@
       <c r="F20" t="n">
         <v>24.1</v>
       </c>
-      <c r="G20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -7859,7 +7807,6 @@
       <c r="F21" t="n">
         <v>20.2</v>
       </c>
-      <c r="G21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -7884,7 +7831,6 @@
       <c r="F22" t="n">
         <v>18</v>
       </c>
-      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -7909,7 +7855,6 @@
       <c r="F23" t="n">
         <v>0.1</v>
       </c>
-      <c r="G23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -7934,7 +7879,6 @@
       <c r="F24" t="n">
         <v>-0.4</v>
       </c>
-      <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -7959,7 +7903,6 @@
       <c r="F25" t="n">
         <v>-0.2</v>
       </c>
-      <c r="G25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -7984,7 +7927,6 @@
       <c r="F26" t="n">
         <v>28.8</v>
       </c>
-      <c r="G26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -8009,7 +7951,6 @@
       <c r="F27" t="n">
         <v>24.4</v>
       </c>
-      <c r="G27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -8034,7 +7975,6 @@
       <c r="F28" t="n">
         <v>20.9</v>
       </c>
-      <c r="G28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -8059,7 +7999,6 @@
       <c r="F29" t="n">
         <v>18</v>
       </c>
-      <c r="G29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -8084,7 +8023,6 @@
       <c r="F30" t="n">
         <v>-0.2</v>
       </c>
-      <c r="G30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -8109,7 +8047,6 @@
       <c r="F31" t="n">
         <v>0.2</v>
       </c>
-      <c r="G31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -8134,7 +8071,6 @@
       <c r="F32" t="n">
         <v>-0.2</v>
       </c>
-      <c r="G32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -8159,7 +8095,6 @@
       <c r="F33" t="n">
         <v>28.5</v>
       </c>
-      <c r="G33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -8184,7 +8119,6 @@
       <c r="F34" t="n">
         <v>23.9</v>
       </c>
-      <c r="G34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -8209,7 +8143,6 @@
       <c r="F35" t="n">
         <v>20.6</v>
       </c>
-      <c r="G35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -8234,7 +8167,6 @@
       <c r="F36" t="n">
         <v>17.9</v>
       </c>
-      <c r="G36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -8259,7 +8191,6 @@
       <c r="F37" t="n">
         <v>-0.2</v>
       </c>
-      <c r="G37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -8284,7 +8215,6 @@
       <c r="F38" t="n">
         <v>0</v>
       </c>
-      <c r="G38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -8309,7 +8239,6 @@
       <c r="F39" t="n">
         <v>0</v>
       </c>
-      <c r="G39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -8334,7 +8263,6 @@
       <c r="F40" t="n">
         <v>28.8</v>
       </c>
-      <c r="G40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -8359,7 +8287,6 @@
       <c r="F41" t="n">
         <v>24.3</v>
       </c>
-      <c r="G41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -8384,7 +8311,6 @@
       <c r="F42" t="n">
         <v>20.6</v>
       </c>
-      <c r="G42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -8409,7 +8335,6 @@
       <c r="F43" t="n">
         <v>18.1</v>
       </c>
-      <c r="G43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -8434,7 +8359,6 @@
       <c r="F44" t="n">
         <v>-0.1</v>
       </c>
-      <c r="G44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -8459,7 +8383,6 @@
       <c r="F45" t="n">
         <v>-0.4</v>
       </c>
-      <c r="G45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -8484,7 +8407,6 @@
       <c r="F46" t="n">
         <v>-1.3</v>
       </c>
-      <c r="G46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -8509,7 +8431,6 @@
       <c r="F47" t="n">
         <v>28.3</v>
       </c>
-      <c r="G47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -8534,7 +8455,6 @@
       <c r="F48" t="n">
         <v>23.9</v>
       </c>
-      <c r="G48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -8559,7 +8479,6 @@
       <c r="F49" t="n">
         <v>20.6</v>
       </c>
-      <c r="G49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -8584,7 +8503,6 @@
       <c r="F50" t="n">
         <v>18.1</v>
       </c>
-      <c r="G50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -8609,7 +8527,6 @@
       <c r="F51" t="n">
         <v>-0.5</v>
       </c>
-      <c r="G51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -8634,7 +8551,6 @@
       <c r="F52" t="n">
         <v>-0.6</v>
       </c>
-      <c r="G52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -8659,7 +8575,6 @@
       <c r="F53" t="n">
         <v>0</v>
       </c>
-      <c r="G53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -8684,7 +8599,6 @@
       <c r="F54" t="n">
         <v>28.4</v>
       </c>
-      <c r="G54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -8709,7 +8623,6 @@
       <c r="F55" t="n">
         <v>24.3</v>
       </c>
-      <c r="G55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -8734,7 +8647,6 @@
       <c r="F56" t="n">
         <v>20.7</v>
       </c>
-      <c r="G56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -8759,7 +8671,6 @@
       <c r="F57" t="n">
         <v>17.8</v>
       </c>
-      <c r="G57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -8784,7 +8695,6 @@
       <c r="F58" t="n">
         <v>-0</v>
       </c>
-      <c r="G58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -8809,7 +8719,6 @@
       <c r="F59" t="n">
         <v>-0.4</v>
       </c>
-      <c r="G59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -8834,7 +8743,6 @@
       <c r="F60" t="n">
         <v>0</v>
       </c>
-      <c r="G60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -8859,7 +8767,6 @@
       <c r="F61" t="n">
         <v>28.8</v>
       </c>
-      <c r="G61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -8884,7 +8791,6 @@
       <c r="F62" t="n">
         <v>23.9</v>
       </c>
-      <c r="G62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -8909,7 +8815,6 @@
       <c r="F63" t="n">
         <v>20.6</v>
       </c>
-      <c r="G63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -8934,7 +8839,6 @@
       <c r="F64" t="n">
         <v>15</v>
       </c>
-      <c r="G64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -8951,15 +8855,14 @@
         <v>2</v>
       </c>
       <c r="D65" t="n">
-        <v>0.3416</v>
+        <v>0.3412</v>
       </c>
       <c r="E65" t="n">
-        <v>0.342</v>
+        <v>0.3425</v>
       </c>
       <c r="F65" t="n">
-        <v>-0.1</v>
-      </c>
-      <c r="G65" t="inlineStr"/>
+        <v>-0.4</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -8976,18 +8879,13 @@
         <v>4</v>
       </c>
       <c r="D66" t="n">
-        <v>0.2438</v>
+        <v>0.1723</v>
       </c>
       <c r="E66" t="n">
-        <v>0.1919</v>
+        <v>0.1727</v>
       </c>
       <c r="F66" t="n">
-        <v>21.3</v>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>rerun pending</t>
-        </is>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="67">
@@ -9005,18 +8903,13 @@
         <v>6</v>
       </c>
       <c r="D67" t="n">
-        <v>0.1683</v>
+        <v>0.1217</v>
       </c>
       <c r="E67" t="n">
-        <v>0.1387</v>
+        <v>0.1223</v>
       </c>
       <c r="F67" t="n">
-        <v>17.6</v>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>rerun pending</t>
-        </is>
+        <v>-0.5</v>
       </c>
     </row>
     <row r="68">
@@ -9034,18 +8927,13 @@
         <v>8</v>
       </c>
       <c r="D68" t="n">
-        <v>0.1473</v>
+        <v>0.1469</v>
       </c>
       <c r="E68" t="n">
-        <v>0.1095</v>
+        <v>0.1051</v>
       </c>
       <c r="F68" t="n">
-        <v>25.7</v>
-      </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>rerun pending</t>
-        </is>
+        <v>28.5</v>
       </c>
     </row>
     <row r="69">
@@ -9063,18 +8951,13 @@
         <v>10</v>
       </c>
       <c r="D69" t="n">
-        <v>0.1186</v>
+        <v>0.1185</v>
       </c>
       <c r="E69" t="n">
-        <v>0.0959</v>
+        <v>0.0901</v>
       </c>
       <c r="F69" t="n">
-        <v>19.1</v>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>rerun pending</t>
-        </is>
+        <v>24</v>
       </c>
     </row>
     <row r="70">
@@ -9095,12 +8978,11 @@
         <v>0.101</v>
       </c>
       <c r="E70" t="n">
-        <v>0.0804</v>
+        <v>0.08019999999999999</v>
       </c>
       <c r="F70" t="n">
-        <v>20.4</v>
-      </c>
-      <c r="G70" t="inlineStr"/>
+        <v>20.6</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -9117,15 +8999,14 @@
         <v>14</v>
       </c>
       <c r="D71" t="n">
-        <v>0.0873</v>
+        <v>0.0872</v>
       </c>
       <c r="E71" t="n">
         <v>0.0716</v>
       </c>
       <c r="F71" t="n">
-        <v>18</v>
-      </c>
-      <c r="G71" t="inlineStr"/>
+        <v>17.9</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -9150,7 +9031,6 @@
       <c r="F72" t="n">
         <v>-0.3</v>
       </c>
-      <c r="G72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -9175,7 +9055,6 @@
       <c r="F73" t="n">
         <v>-0.7</v>
       </c>
-      <c r="G73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -9200,7 +9079,6 @@
       <c r="F74" t="n">
         <v>-0.2</v>
       </c>
-      <c r="G74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -9225,7 +9103,6 @@
       <c r="F75" t="n">
         <v>28.6</v>
       </c>
-      <c r="G75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -9250,7 +9127,6 @@
       <c r="F76" t="n">
         <v>24.2</v>
       </c>
-      <c r="G76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -9275,7 +9151,6 @@
       <c r="F77" t="n">
         <v>20.5</v>
       </c>
-      <c r="G77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -9300,7 +9175,6 @@
       <c r="F78" t="n">
         <v>18</v>
       </c>
-      <c r="G78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -9325,7 +9199,6 @@
       <c r="F79" t="n">
         <v>-0.5</v>
       </c>
-      <c r="G79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -9350,7 +9223,6 @@
       <c r="F80" t="n">
         <v>0</v>
       </c>
-      <c r="G80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -9375,7 +9247,6 @@
       <c r="F81" t="n">
         <v>0.1</v>
       </c>
-      <c r="G81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -9400,7 +9271,6 @@
       <c r="F82" t="n">
         <v>28.3</v>
       </c>
-      <c r="G82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -9425,7 +9295,6 @@
       <c r="F83" t="n">
         <v>24.2</v>
       </c>
-      <c r="G83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -9450,7 +9319,6 @@
       <c r="F84" t="n">
         <v>20.6</v>
       </c>
-      <c r="G84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -9475,7 +9343,6 @@
       <c r="F85" t="n">
         <v>18</v>
       </c>
-      <c r="G85" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Re-measure five suspect Equal/Adaptive cells; add diagnostics to tables and text
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T6gEewJ8YaCdmnsfS34RJd
</commit_message>
<xml_diff>
--- a/results/final_results.xlsx
+++ b/results/final_results.xlsx
@@ -19,6 +19,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EqAd unified (LBG+Total)" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EqAd summary" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Throughput" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Remeasure 5 cells (raw)" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Remeasure summary" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6703,6 +6705,2039 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>np</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>run</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>equal_lbg_s</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>adaptive_lbg_s</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>P_speed_mean</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>E_speed_mean</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>E_speed_min</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>P_vectors_rank0</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>E_vectors_lastrank</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>lung_ct2_img</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.0448</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.0355</v>
+      </c>
+      <c r="F2" t="n">
+        <v>276</v>
+      </c>
+      <c r="G2" t="n">
+        <v>176.7</v>
+      </c>
+      <c r="H2" t="n">
+        <v>176.4</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1669</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>lung_ct2_img</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>12</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.0448</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.0356</v>
+      </c>
+      <c r="F3" t="n">
+        <v>275.2</v>
+      </c>
+      <c r="G3" t="n">
+        <v>176.6</v>
+      </c>
+      <c r="H3" t="n">
+        <v>176.5</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1654</v>
+      </c>
+      <c r="J3" t="n">
+        <v>1069</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>lung_ct2_img</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>12</v>
+      </c>
+      <c r="C4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.0448</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.0354</v>
+      </c>
+      <c r="F4" t="n">
+        <v>275.5</v>
+      </c>
+      <c r="G4" t="n">
+        <v>175</v>
+      </c>
+      <c r="H4" t="n">
+        <v>170.8</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1665</v>
+      </c>
+      <c r="J4" t="n">
+        <v>1073</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>lung_ct2_img</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>12</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.0448</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.0356</v>
+      </c>
+      <c r="F5" t="n">
+        <v>275</v>
+      </c>
+      <c r="G5" t="n">
+        <v>176.6</v>
+      </c>
+      <c r="H5" t="n">
+        <v>176.2</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1656</v>
+      </c>
+      <c r="J5" t="n">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>lung_ct2_img</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>12</v>
+      </c>
+      <c r="C6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.0448</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.0354</v>
+      </c>
+      <c r="F6" t="n">
+        <v>275.3</v>
+      </c>
+      <c r="G6" t="n">
+        <v>176.6</v>
+      </c>
+      <c r="H6" t="n">
+        <v>176.4</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1670</v>
+      </c>
+      <c r="J6" t="n">
+        <v>1069</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>lung_ct2_img</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>12</v>
+      </c>
+      <c r="C7" t="n">
+        <v>6</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.0448</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.0355</v>
+      </c>
+      <c r="F7" t="n">
+        <v>275.8</v>
+      </c>
+      <c r="G7" t="n">
+        <v>176.6</v>
+      </c>
+      <c r="H7" t="n">
+        <v>176.3</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1668</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>lung_ct2_img</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>12</v>
+      </c>
+      <c r="C8" t="n">
+        <v>7</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.0448</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.0354</v>
+      </c>
+      <c r="F8" t="n">
+        <v>276.1</v>
+      </c>
+      <c r="G8" t="n">
+        <v>176.7</v>
+      </c>
+      <c r="H8" t="n">
+        <v>176.3</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1667</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>lung_ct2_img</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>12</v>
+      </c>
+      <c r="C9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.0448</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.0356</v>
+      </c>
+      <c r="F9" t="n">
+        <v>275</v>
+      </c>
+      <c r="G9" t="n">
+        <v>176.6</v>
+      </c>
+      <c r="H9" t="n">
+        <v>176.3</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1671</v>
+      </c>
+      <c r="J9" t="n">
+        <v>1069</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>lung_ct2_img</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>12</v>
+      </c>
+      <c r="C10" t="n">
+        <v>9</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.0448</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.0355</v>
+      </c>
+      <c r="F10" t="n">
+        <v>275.6</v>
+      </c>
+      <c r="G10" t="n">
+        <v>176.5</v>
+      </c>
+      <c r="H10" t="n">
+        <v>176.3</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1661</v>
+      </c>
+      <c r="J10" t="n">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>lung_ct2_img</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>12</v>
+      </c>
+      <c r="C11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.0447</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.0355</v>
+      </c>
+      <c r="F11" t="n">
+        <v>275.2</v>
+      </c>
+      <c r="G11" t="n">
+        <v>176.6</v>
+      </c>
+      <c r="H11" t="n">
+        <v>176.4</v>
+      </c>
+      <c r="I11" t="n">
+        <v>1670</v>
+      </c>
+      <c r="J11" t="n">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>lung_ct2_img</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>14</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.0387</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.0318</v>
+      </c>
+      <c r="F12" t="n">
+        <v>275.1</v>
+      </c>
+      <c r="G12" t="n">
+        <v>176.5</v>
+      </c>
+      <c r="H12" t="n">
+        <v>176.4</v>
+      </c>
+      <c r="I12" t="n">
+        <v>1464</v>
+      </c>
+      <c r="J12" t="n">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>lung_ct2_img</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>14</v>
+      </c>
+      <c r="C13" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.0388</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.0322</v>
+      </c>
+      <c r="F13" t="n">
+        <v>274.6</v>
+      </c>
+      <c r="G13" t="n">
+        <v>176.5</v>
+      </c>
+      <c r="H13" t="n">
+        <v>176.4</v>
+      </c>
+      <c r="I13" t="n">
+        <v>1465</v>
+      </c>
+      <c r="J13" t="n">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>lung_ct2_img</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>14</v>
+      </c>
+      <c r="C14" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.0388</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.0349</v>
+      </c>
+      <c r="F14" t="n">
+        <v>275.1</v>
+      </c>
+      <c r="G14" t="n">
+        <v>176.4</v>
+      </c>
+      <c r="H14" t="n">
+        <v>176.3</v>
+      </c>
+      <c r="I14" t="n">
+        <v>1480</v>
+      </c>
+      <c r="J14" t="n">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>lung_ct2_img</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.0388</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.0317</v>
+      </c>
+      <c r="F15" t="n">
+        <v>275.6</v>
+      </c>
+      <c r="G15" t="n">
+        <v>176.5</v>
+      </c>
+      <c r="H15" t="n">
+        <v>176.3</v>
+      </c>
+      <c r="I15" t="n">
+        <v>1478</v>
+      </c>
+      <c r="J15" t="n">
+        <v>943</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>lung_ct2_img</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>14</v>
+      </c>
+      <c r="C16" t="n">
+        <v>5</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.0387</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.0319</v>
+      </c>
+      <c r="F16" t="n">
+        <v>273.5</v>
+      </c>
+      <c r="G16" t="n">
+        <v>175.2</v>
+      </c>
+      <c r="H16" t="n">
+        <v>170.3</v>
+      </c>
+      <c r="I16" t="n">
+        <v>1480</v>
+      </c>
+      <c r="J16" t="n">
+        <v>952</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>lung_ct2_img</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>14</v>
+      </c>
+      <c r="C17" t="n">
+        <v>6</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.0388</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.0321</v>
+      </c>
+      <c r="F17" t="n">
+        <v>274.8</v>
+      </c>
+      <c r="G17" t="n">
+        <v>176.5</v>
+      </c>
+      <c r="H17" t="n">
+        <v>176.3</v>
+      </c>
+      <c r="I17" t="n">
+        <v>1477</v>
+      </c>
+      <c r="J17" t="n">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>lung_ct2_img</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>14</v>
+      </c>
+      <c r="C18" t="n">
+        <v>7</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.0387</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.0317</v>
+      </c>
+      <c r="F18" t="n">
+        <v>274.6</v>
+      </c>
+      <c r="G18" t="n">
+        <v>176.5</v>
+      </c>
+      <c r="H18" t="n">
+        <v>176.4</v>
+      </c>
+      <c r="I18" t="n">
+        <v>1480</v>
+      </c>
+      <c r="J18" t="n">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>lung_ct2_img</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>14</v>
+      </c>
+      <c r="C19" t="n">
+        <v>8</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.0388</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.0318</v>
+      </c>
+      <c r="F19" t="n">
+        <v>275.3</v>
+      </c>
+      <c r="G19" t="n">
+        <v>176.5</v>
+      </c>
+      <c r="H19" t="n">
+        <v>176.4</v>
+      </c>
+      <c r="I19" t="n">
+        <v>1478</v>
+      </c>
+      <c r="J19" t="n">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>lung_ct2_img</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>14</v>
+      </c>
+      <c r="C20" t="n">
+        <v>9</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.0387</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.0318</v>
+      </c>
+      <c r="F20" t="n">
+        <v>275.5</v>
+      </c>
+      <c r="G20" t="n">
+        <v>176.5</v>
+      </c>
+      <c r="H20" t="n">
+        <v>176.4</v>
+      </c>
+      <c r="I20" t="n">
+        <v>1475</v>
+      </c>
+      <c r="J20" t="n">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>lung_ct2_img</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>14</v>
+      </c>
+      <c r="C21" t="n">
+        <v>10</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.0388</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.0319</v>
+      </c>
+      <c r="F21" t="n">
+        <v>275.1</v>
+      </c>
+      <c r="G21" t="n">
+        <v>176.5</v>
+      </c>
+      <c r="H21" t="n">
+        <v>176.4</v>
+      </c>
+      <c r="I21" t="n">
+        <v>1471</v>
+      </c>
+      <c r="J21" t="n">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>chest_xray2_img</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>14</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0.0313</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0.0256</v>
+      </c>
+      <c r="F22" t="n">
+        <v>275.1</v>
+      </c>
+      <c r="G22" t="n">
+        <v>176.5</v>
+      </c>
+      <c r="H22" t="n">
+        <v>176.4</v>
+      </c>
+      <c r="I22" t="n">
+        <v>1478</v>
+      </c>
+      <c r="J22" t="n">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>chest_xray2_img</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>14</v>
+      </c>
+      <c r="C23" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0.0313</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0.0257</v>
+      </c>
+      <c r="F23" t="n">
+        <v>275.7</v>
+      </c>
+      <c r="G23" t="n">
+        <v>176.5</v>
+      </c>
+      <c r="H23" t="n">
+        <v>176.3</v>
+      </c>
+      <c r="I23" t="n">
+        <v>1476</v>
+      </c>
+      <c r="J23" t="n">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>chest_xray2_img</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>14</v>
+      </c>
+      <c r="C24" t="n">
+        <v>3</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0.0311</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.0258</v>
+      </c>
+      <c r="F24" t="n">
+        <v>275</v>
+      </c>
+      <c r="G24" t="n">
+        <v>176.5</v>
+      </c>
+      <c r="H24" t="n">
+        <v>176.4</v>
+      </c>
+      <c r="I24" t="n">
+        <v>1479</v>
+      </c>
+      <c r="J24" t="n">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>chest_xray2_img</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>14</v>
+      </c>
+      <c r="C25" t="n">
+        <v>4</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0.0313</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.0258</v>
+      </c>
+      <c r="F25" t="n">
+        <v>275.3</v>
+      </c>
+      <c r="G25" t="n">
+        <v>176.5</v>
+      </c>
+      <c r="H25" t="n">
+        <v>176.4</v>
+      </c>
+      <c r="I25" t="n">
+        <v>1477</v>
+      </c>
+      <c r="J25" t="n">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>chest_xray2_img</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>14</v>
+      </c>
+      <c r="C26" t="n">
+        <v>5</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0.0313</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.0256</v>
+      </c>
+      <c r="F26" t="n">
+        <v>275.6</v>
+      </c>
+      <c r="G26" t="n">
+        <v>176.6</v>
+      </c>
+      <c r="H26" t="n">
+        <v>176.4</v>
+      </c>
+      <c r="I26" t="n">
+        <v>1468</v>
+      </c>
+      <c r="J26" t="n">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>chest_xray2_img</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>14</v>
+      </c>
+      <c r="C27" t="n">
+        <v>6</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.0312</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.0256</v>
+      </c>
+      <c r="F27" t="n">
+        <v>274.7</v>
+      </c>
+      <c r="G27" t="n">
+        <v>176.5</v>
+      </c>
+      <c r="H27" t="n">
+        <v>176.3</v>
+      </c>
+      <c r="I27" t="n">
+        <v>1466</v>
+      </c>
+      <c r="J27" t="n">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>chest_xray2_img</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>14</v>
+      </c>
+      <c r="C28" t="n">
+        <v>7</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0.0313</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.0257</v>
+      </c>
+      <c r="F28" t="n">
+        <v>274.5</v>
+      </c>
+      <c r="G28" t="n">
+        <v>176.5</v>
+      </c>
+      <c r="H28" t="n">
+        <v>176.4</v>
+      </c>
+      <c r="I28" t="n">
+        <v>1472</v>
+      </c>
+      <c r="J28" t="n">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>chest_xray2_img</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>14</v>
+      </c>
+      <c r="C29" t="n">
+        <v>8</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0.0312</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.0255</v>
+      </c>
+      <c r="F29" t="n">
+        <v>275.8</v>
+      </c>
+      <c r="G29" t="n">
+        <v>176.5</v>
+      </c>
+      <c r="H29" t="n">
+        <v>176.3</v>
+      </c>
+      <c r="I29" t="n">
+        <v>1476</v>
+      </c>
+      <c r="J29" t="n">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>chest_xray2_img</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>14</v>
+      </c>
+      <c r="C30" t="n">
+        <v>9</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0.0311</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0.0257</v>
+      </c>
+      <c r="F30" t="n">
+        <v>275.9</v>
+      </c>
+      <c r="G30" t="n">
+        <v>176.6</v>
+      </c>
+      <c r="H30" t="n">
+        <v>176.5</v>
+      </c>
+      <c r="I30" t="n">
+        <v>1476</v>
+      </c>
+      <c r="J30" t="n">
+        <v>943</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>chest_xray2_img</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>14</v>
+      </c>
+      <c r="C31" t="n">
+        <v>10</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0.0313</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0.0255</v>
+      </c>
+      <c r="F31" t="n">
+        <v>274.6</v>
+      </c>
+      <c r="G31" t="n">
+        <v>176.6</v>
+      </c>
+      <c r="H31" t="n">
+        <v>176.5</v>
+      </c>
+      <c r="I31" t="n">
+        <v>1479</v>
+      </c>
+      <c r="J31" t="n">
+        <v>946</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>mammo2_img</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>14</v>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0.0278</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0.0228</v>
+      </c>
+      <c r="F32" t="n">
+        <v>275.2</v>
+      </c>
+      <c r="G32" t="n">
+        <v>176.6</v>
+      </c>
+      <c r="H32" t="n">
+        <v>176.5</v>
+      </c>
+      <c r="I32" t="n">
+        <v>1471</v>
+      </c>
+      <c r="J32" t="n">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>mammo2_img</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>14</v>
+      </c>
+      <c r="C33" t="n">
+        <v>2</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0.0278</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0.0228</v>
+      </c>
+      <c r="F33" t="n">
+        <v>275.5</v>
+      </c>
+      <c r="G33" t="n">
+        <v>176.6</v>
+      </c>
+      <c r="H33" t="n">
+        <v>176.4</v>
+      </c>
+      <c r="I33" t="n">
+        <v>1457</v>
+      </c>
+      <c r="J33" t="n">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>mammo2_img</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>14</v>
+      </c>
+      <c r="C34" t="n">
+        <v>3</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0.0278</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0.0227</v>
+      </c>
+      <c r="F34" t="n">
+        <v>275.9</v>
+      </c>
+      <c r="G34" t="n">
+        <v>176.6</v>
+      </c>
+      <c r="H34" t="n">
+        <v>176.6</v>
+      </c>
+      <c r="I34" t="n">
+        <v>1475</v>
+      </c>
+      <c r="J34" t="n">
+        <v>943</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>mammo2_img</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>14</v>
+      </c>
+      <c r="C35" t="n">
+        <v>4</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0.0278</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0.0227</v>
+      </c>
+      <c r="F35" t="n">
+        <v>275.4</v>
+      </c>
+      <c r="G35" t="n">
+        <v>176.5</v>
+      </c>
+      <c r="H35" t="n">
+        <v>176.4</v>
+      </c>
+      <c r="I35" t="n">
+        <v>1477</v>
+      </c>
+      <c r="J35" t="n">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>mammo2_img</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>14</v>
+      </c>
+      <c r="C36" t="n">
+        <v>5</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0.0278</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0.0228</v>
+      </c>
+      <c r="F36" t="n">
+        <v>274.5</v>
+      </c>
+      <c r="G36" t="n">
+        <v>176.5</v>
+      </c>
+      <c r="H36" t="n">
+        <v>176.4</v>
+      </c>
+      <c r="I36" t="n">
+        <v>1480</v>
+      </c>
+      <c r="J36" t="n">
+        <v>946</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>mammo2_img</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>14</v>
+      </c>
+      <c r="C37" t="n">
+        <v>6</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0.0278</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0.0228</v>
+      </c>
+      <c r="F37" t="n">
+        <v>274.8</v>
+      </c>
+      <c r="G37" t="n">
+        <v>176.5</v>
+      </c>
+      <c r="H37" t="n">
+        <v>176.4</v>
+      </c>
+      <c r="I37" t="n">
+        <v>1480</v>
+      </c>
+      <c r="J37" t="n">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>mammo2_img</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>14</v>
+      </c>
+      <c r="C38" t="n">
+        <v>7</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0.0278</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0.0228</v>
+      </c>
+      <c r="F38" t="n">
+        <v>276.1</v>
+      </c>
+      <c r="G38" t="n">
+        <v>176.5</v>
+      </c>
+      <c r="H38" t="n">
+        <v>176.3</v>
+      </c>
+      <c r="I38" t="n">
+        <v>1475</v>
+      </c>
+      <c r="J38" t="n">
+        <v>943</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>mammo2_img</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>14</v>
+      </c>
+      <c r="C39" t="n">
+        <v>8</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0.0278</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0.0228</v>
+      </c>
+      <c r="F39" t="n">
+        <v>275.7</v>
+      </c>
+      <c r="G39" t="n">
+        <v>176.5</v>
+      </c>
+      <c r="H39" t="n">
+        <v>176.4</v>
+      </c>
+      <c r="I39" t="n">
+        <v>1477</v>
+      </c>
+      <c r="J39" t="n">
+        <v>943</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>mammo2_img</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>14</v>
+      </c>
+      <c r="C40" t="n">
+        <v>9</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0.0278</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0.0229</v>
+      </c>
+      <c r="F40" t="n">
+        <v>274.1</v>
+      </c>
+      <c r="G40" t="n">
+        <v>176.5</v>
+      </c>
+      <c r="H40" t="n">
+        <v>176.3</v>
+      </c>
+      <c r="I40" t="n">
+        <v>1481</v>
+      </c>
+      <c r="J40" t="n">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>mammo2_img</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>14</v>
+      </c>
+      <c r="C41" t="n">
+        <v>10</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0.0278</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0.0236</v>
+      </c>
+      <c r="F41" t="n">
+        <v>275.2</v>
+      </c>
+      <c r="G41" t="n">
+        <v>175.3</v>
+      </c>
+      <c r="H41" t="n">
+        <v>166.6</v>
+      </c>
+      <c r="I41" t="n">
+        <v>1482</v>
+      </c>
+      <c r="J41" t="n">
+        <v>894</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>peppers_img</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>8</v>
+      </c>
+      <c r="C42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" t="n">
+        <v>0.0629</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0.0453</v>
+      </c>
+      <c r="F42" t="n">
+        <v>275.1</v>
+      </c>
+      <c r="G42" t="n">
+        <v>176.8</v>
+      </c>
+      <c r="H42" t="n">
+        <v>176.7</v>
+      </c>
+      <c r="I42" t="n">
+        <v>2258</v>
+      </c>
+      <c r="J42" t="n">
+        <v>1447</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>peppers_img</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>8</v>
+      </c>
+      <c r="C43" t="n">
+        <v>2</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0.063</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="F43" t="n">
+        <v>274.8</v>
+      </c>
+      <c r="G43" t="n">
+        <v>177</v>
+      </c>
+      <c r="H43" t="n">
+        <v>177</v>
+      </c>
+      <c r="I43" t="n">
+        <v>2241</v>
+      </c>
+      <c r="J43" t="n">
+        <v>1448</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>peppers_img</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>8</v>
+      </c>
+      <c r="C44" t="n">
+        <v>3</v>
+      </c>
+      <c r="D44" t="n">
+        <v>0.0629</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0.0456</v>
+      </c>
+      <c r="F44" t="n">
+        <v>275.4</v>
+      </c>
+      <c r="G44" t="n">
+        <v>176.4</v>
+      </c>
+      <c r="H44" t="n">
+        <v>175.9</v>
+      </c>
+      <c r="I44" t="n">
+        <v>2236</v>
+      </c>
+      <c r="J44" t="n">
+        <v>1446</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>peppers_img</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>8</v>
+      </c>
+      <c r="C45" t="n">
+        <v>4</v>
+      </c>
+      <c r="D45" t="n">
+        <v>0.0626</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="F45" t="n">
+        <v>274.5</v>
+      </c>
+      <c r="G45" t="n">
+        <v>176.9</v>
+      </c>
+      <c r="H45" t="n">
+        <v>176.8</v>
+      </c>
+      <c r="I45" t="n">
+        <v>2262</v>
+      </c>
+      <c r="J45" t="n">
+        <v>1448</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>peppers_img</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>8</v>
+      </c>
+      <c r="C46" t="n">
+        <v>5</v>
+      </c>
+      <c r="D46" t="n">
+        <v>0.0624</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0.0445</v>
+      </c>
+      <c r="F46" t="n">
+        <v>275.5</v>
+      </c>
+      <c r="G46" t="n">
+        <v>177</v>
+      </c>
+      <c r="H46" t="n">
+        <v>176.9</v>
+      </c>
+      <c r="I46" t="n">
+        <v>2234</v>
+      </c>
+      <c r="J46" t="n">
+        <v>1445</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>peppers_img</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>8</v>
+      </c>
+      <c r="C47" t="n">
+        <v>6</v>
+      </c>
+      <c r="D47" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0.0445</v>
+      </c>
+      <c r="F47" t="n">
+        <v>275.7</v>
+      </c>
+      <c r="G47" t="n">
+        <v>177</v>
+      </c>
+      <c r="H47" t="n">
+        <v>177</v>
+      </c>
+      <c r="I47" t="n">
+        <v>2255</v>
+      </c>
+      <c r="J47" t="n">
+        <v>1444</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>peppers_img</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>8</v>
+      </c>
+      <c r="C48" t="n">
+        <v>7</v>
+      </c>
+      <c r="D48" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0.0445</v>
+      </c>
+      <c r="F48" t="n">
+        <v>275.3</v>
+      </c>
+      <c r="G48" t="n">
+        <v>176.9</v>
+      </c>
+      <c r="H48" t="n">
+        <v>176.7</v>
+      </c>
+      <c r="I48" t="n">
+        <v>2237</v>
+      </c>
+      <c r="J48" t="n">
+        <v>1444</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>peppers_img</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>8</v>
+      </c>
+      <c r="C49" t="n">
+        <v>8</v>
+      </c>
+      <c r="D49" t="n">
+        <v>0.0624</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0.0445</v>
+      </c>
+      <c r="F49" t="n">
+        <v>275.9</v>
+      </c>
+      <c r="G49" t="n">
+        <v>177</v>
+      </c>
+      <c r="H49" t="n">
+        <v>177</v>
+      </c>
+      <c r="I49" t="n">
+        <v>2253</v>
+      </c>
+      <c r="J49" t="n">
+        <v>1443</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>peppers_img</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>8</v>
+      </c>
+      <c r="C50" t="n">
+        <v>9</v>
+      </c>
+      <c r="D50" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="E50" t="n">
+        <v>0.0445</v>
+      </c>
+      <c r="F50" t="n">
+        <v>275.7</v>
+      </c>
+      <c r="G50" t="n">
+        <v>176.9</v>
+      </c>
+      <c r="H50" t="n">
+        <v>176.8</v>
+      </c>
+      <c r="I50" t="n">
+        <v>2254</v>
+      </c>
+      <c r="J50" t="n">
+        <v>1444</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>peppers_img</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>8</v>
+      </c>
+      <c r="C51" t="n">
+        <v>10</v>
+      </c>
+      <c r="D51" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="E51" t="n">
+        <v>0.0445</v>
+      </c>
+      <c r="F51" t="n">
+        <v>275</v>
+      </c>
+      <c r="G51" t="n">
+        <v>176.9</v>
+      </c>
+      <c r="H51" t="n">
+        <v>176.8</v>
+      </c>
+      <c r="I51" t="n">
+        <v>2260</v>
+      </c>
+      <c r="J51" t="n">
+        <v>1447</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>np</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>equal_median_10runs</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>adaptive_median_10runs</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>gain_pct_10runs</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>unified_equal</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>unified_adaptive</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>unified_gain_pct</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>session1_adaptive</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>session1_gain_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>lung_ct2_img</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.0448</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.0355</v>
+      </c>
+      <c r="E2" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.0448</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.0378</v>
+      </c>
+      <c r="H2" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.0354</v>
+      </c>
+      <c r="J2" t="n">
+        <v>20.6</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>lung_ct2_img</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>14</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.0388</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.0318</v>
+      </c>
+      <c r="E3" t="n">
+        <v>18</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.0387</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.0337</v>
+      </c>
+      <c r="H3" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.0317</v>
+      </c>
+      <c r="J3" t="n">
+        <v>18.1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>chest_xray2_img</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>14</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.0313</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.0256</v>
+      </c>
+      <c r="E4" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.0312</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.0274</v>
+      </c>
+      <c r="H4" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.0256</v>
+      </c>
+      <c r="J4" t="n">
+        <v>17.9</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>mammo2_img</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>14</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.0278</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.0228</v>
+      </c>
+      <c r="E5" t="n">
+        <v>18</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.0293</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.0251</v>
+      </c>
+      <c r="H5" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.0227</v>
+      </c>
+      <c r="J5" t="n">
+        <v>18.1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>peppers_img</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>8</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.0445</v>
+      </c>
+      <c r="E6" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.0624</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.0461</v>
+      </c>
+      <c r="H6" t="n">
+        <v>26.1</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.0446</v>
+      </c>
+      <c r="J6" t="n">
+        <v>28.8</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Ten alternated Equal/Adaptive runs per cell with the calibrated rank speeds recorded (diag_adaptive.sh). Medians use the lower-median rule of the scripts.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add entropy results (grayscale) to tables
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T6gEewJ8YaCdmnsfS34RJd
</commit_message>
<xml_diff>
--- a/results/final_results.xlsx
+++ b/results/final_results.xlsx
@@ -21,6 +21,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Throughput" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Remeasure 5 cells (raw)" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Remeasure summary" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Entropy" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -8738,6 +8739,326 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>H_index_bits</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>H_delta_bits</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>delta_reduction_bits</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>huffman_data_bytes</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>huffman_bits_per_index</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>gap_vs_H_delta_bits</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>saving_vs_6bit_fixed_pct</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>system_CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Lena</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>5.393</v>
+      </c>
+      <c r="C2" t="n">
+        <v>4.665</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.728</v>
+      </c>
+      <c r="E2" t="n">
+        <v>9648</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4.711</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.046</v>
+      </c>
+      <c r="H2" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="I2" t="n">
+        <v>23.5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Boat</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>5.237</v>
+      </c>
+      <c r="C3" t="n">
+        <v>4.061</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1.176</v>
+      </c>
+      <c r="E3" t="n">
+        <v>8359</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4.082</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="H3" t="n">
+        <v>32</v>
+      </c>
+      <c r="I3" t="n">
+        <v>26.54</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Cameraman</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>5.165</v>
+      </c>
+      <c r="C4" t="n">
+        <v>3.682</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1.483</v>
+      </c>
+      <c r="E4" t="n">
+        <v>7584</v>
+      </c>
+      <c r="F4" t="n">
+        <v>3.703</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="H4" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="I4" t="n">
+        <v>28.88</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Peppers</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>5.396</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4.365</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1.031</v>
+      </c>
+      <c r="E5" t="n">
+        <v>9078</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4.433</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.068</v>
+      </c>
+      <c r="H5" t="n">
+        <v>26.1</v>
+      </c>
+      <c r="I5" t="n">
+        <v>24.75</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Chest X-ray</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5.63</v>
+      </c>
+      <c r="C6" t="n">
+        <v>4.724</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.906</v>
+      </c>
+      <c r="E6" t="n">
+        <v>9721</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4.747</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="H6" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="I6" t="n">
+        <v>23.39</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Mammogram</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>5.465</v>
+      </c>
+      <c r="C7" t="n">
+        <v>3.332</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2.133</v>
+      </c>
+      <c r="E7" t="n">
+        <v>6853</v>
+      </c>
+      <c r="F7" t="n">
+        <v>3.346</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="H7" t="n">
+        <v>44.2</v>
+      </c>
+      <c r="I7" t="n">
+        <v>31.56</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Lung CT</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>4.581</v>
+      </c>
+      <c r="C8" t="n">
+        <v>4.394</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.187</v>
+      </c>
+      <c r="E8" t="n">
+        <v>9141</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4.463</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.06900000000000001</v>
+      </c>
+      <c r="H8" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="I8" t="n">
+        <v>24.63</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Brain MRI</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>4.084</v>
+      </c>
+      <c r="C9" t="n">
+        <v>3.018</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1.066</v>
+      </c>
+      <c r="E9" t="n">
+        <v>6316</v>
+      </c>
+      <c r="F9" t="n">
+        <v>3.084</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.066</v>
+      </c>
+      <c r="H9" t="n">
+        <v>48.6</v>
+      </c>
+      <c r="I9" t="n">
+        <v>33.49</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add correctness results (12 images x 4 configurations) and section 4.8 text
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T6gEewJ8YaCdmnsfS34RJd
</commit_message>
<xml_diff>
--- a/results/final_results.xlsx
+++ b/results/final_results.xlsx
@@ -22,6 +22,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Remeasure 5 cells (raw)" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Remeasure summary" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Entropy" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Correctness" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -9059,6 +9060,576 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>mode</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>CR MSE PSNR SSIM iters: sequential</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>P=4 (Equal, default)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>P=14 (Adaptive, default)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>P=14 (Equal, forced)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>metrics identical</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>reconstruction MD5 identical</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>23.50 58.77 30.44 0.8431 160</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>23.50 58.77 30.44 0.8431 160</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>23.50 58.77 30.44 0.8431 160</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>23.50 58.77 30.44 0.8431 160</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>boat_img</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>26.54 70.46 29.65 0.8522 151</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>26.54 70.46 29.65 0.8522 151</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>26.54 70.46 29.65 0.8522 151</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>26.54 70.46 29.65 0.8522 151</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>cameraman_img</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>28.88 56.66 30.60 0.9031 155</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>28.88 56.66 30.60 0.9031 155</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>28.88 56.66 30.60 0.9031 155</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>28.88 56.66 30.60 0.9031 155</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>peppers_img</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>24.75 61.51 30.24 0.7875 132</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>24.75 61.51 30.24 0.7875 132</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>24.75 61.51 30.24 0.7875 132</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>24.75 61.51 30.24 0.7875 132</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>chest_xray2_img</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>23.39 25.05 34.14 0.8890 125</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>23.39 25.05 34.14 0.8890 125</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>23.39 25.05 34.14 0.8890 125</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>23.39 25.05 34.14 0.8890 125</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>mammo2_img</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>31.56 13.81 36.73 0.9392 98</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>31.56 13.81 36.73 0.9392 98</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>31.56 13.81 36.73 0.9392 98</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>31.56 13.81 36.73 0.9392 98</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>lung_ct2_img</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>24.63 83.81 28.90 0.8666 197</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>24.63 83.81 28.90 0.8666 197</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>24.63 83.81 28.90 0.8666 197</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>24.63 83.81 28.90 0.8666 197</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>brain_mri2_img</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>33.49 23.08 34.50 0.9474 142</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>33.49 23.08 34.50 0.9474 142</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>33.49 23.08 34.50 0.9474 142</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>33.49 23.08 34.50 0.9474 142</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>lena_color</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>24.00 75.25 29.37 0.7733 476</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>24.00 75.25 29.37 0.7733 476</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>24.00 75.25 29.37 0.7733 476</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>24.00 75.25 29.37 0.7733 476</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>retina2_color</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>34.07 5.97 40.37 0.9541 493</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>34.07 5.97 40.37 0.9541 493</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>34.07 5.97 40.37 0.9541 493</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>34.07 5.97 40.37 0.9541 493</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>brain_pet3_color</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>25.05 94.94 28.36 0.8793 495</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>25.05 94.94 28.36 0.8793 495</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>25.05 94.94 28.36 0.8793 495</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>25.05 94.94 28.36 0.8793 495</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>brain_pet4_color</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>22.24 53.82 30.82 0.8995 502</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>22.24 53.82 30.82 0.8995 502</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>22.24 53.82 30.82 0.8995 502</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>22.24 53.82 30.82 0.8995 502</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add Block/K study, index-coding and JPEG/JPEG2000 reference tables and data
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T6gEewJ8YaCdmnsfS34RJd
</commit_message>
<xml_diff>
--- a/results/final_results.xlsx
+++ b/results/final_results.xlsx
@@ -23,6 +23,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Remeasure summary" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Entropy" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Correctness" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Param study" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baselines JPEG-J2K" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Index coding" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -9630,6 +9633,2250 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>variant</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>block</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>PSNR_dB</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>SSIM</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>system_CR</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>LBG_iters</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>LBG_time_median_s</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2x2/K64</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" t="n">
+        <v>64</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Lena</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>34.71</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.9214</v>
+      </c>
+      <c r="G2" t="n">
+        <v>6.97</v>
+      </c>
+      <c r="H2" t="n">
+        <v>204</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.4406</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2x2/K64</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="n">
+        <v>64</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Boat</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>33.55</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.9273</v>
+      </c>
+      <c r="G3" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="H3" t="n">
+        <v>285</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.5679</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2x2/K64</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="n">
+        <v>64</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Cameraman</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>35.81</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.9647</v>
+      </c>
+      <c r="G4" t="n">
+        <v>8.56</v>
+      </c>
+      <c r="H4" t="n">
+        <v>203</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.49</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2x2/K64</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" t="n">
+        <v>64</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Peppers</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>33.58</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.872</v>
+      </c>
+      <c r="G5" t="n">
+        <v>7.18</v>
+      </c>
+      <c r="H5" t="n">
+        <v>108</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.2577</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2x2/K64</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" t="n">
+        <v>64</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Chest_X-ray</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>38.33</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.9560999999999999</v>
+      </c>
+      <c r="G6" t="n">
+        <v>7.34</v>
+      </c>
+      <c r="H6" t="n">
+        <v>116</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.2554</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2x2/K64</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" t="n">
+        <v>64</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Mammogram</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>41.26</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.9772</v>
+      </c>
+      <c r="G7" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="H7" t="n">
+        <v>109</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.3251</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2x2/K64</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" t="n">
+        <v>64</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Lung_CT</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>34.09</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.9545</v>
+      </c>
+      <c r="G8" t="n">
+        <v>7.19</v>
+      </c>
+      <c r="H8" t="n">
+        <v>212</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.4465</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2x2/K64</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" t="n">
+        <v>64</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Brain_MRI</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>39.91</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.9836</v>
+      </c>
+      <c r="G9" t="n">
+        <v>10.67</v>
+      </c>
+      <c r="H9" t="n">
+        <v>192</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.5589</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>4x4/K64</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>4</v>
+      </c>
+      <c r="C10" t="n">
+        <v>64</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Lena</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>30.44</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.8431</v>
+      </c>
+      <c r="G10" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="H10" t="n">
+        <v>160</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.2653</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>4x4/K64</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>4</v>
+      </c>
+      <c r="C11" t="n">
+        <v>64</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Boat</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>29.65</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.8522</v>
+      </c>
+      <c r="G11" t="n">
+        <v>26.54</v>
+      </c>
+      <c r="H11" t="n">
+        <v>151</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.2326</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>4x4/K64</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" t="n">
+        <v>64</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Cameraman</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.9031</v>
+      </c>
+      <c r="G12" t="n">
+        <v>28.88</v>
+      </c>
+      <c r="H12" t="n">
+        <v>155</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.2372</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>4x4/K64</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>4</v>
+      </c>
+      <c r="C13" t="n">
+        <v>64</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Peppers</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>30.24</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.7875</v>
+      </c>
+      <c r="G13" t="n">
+        <v>24.75</v>
+      </c>
+      <c r="H13" t="n">
+        <v>132</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.2798</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>4x4/K64</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>4</v>
+      </c>
+      <c r="C14" t="n">
+        <v>64</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Chest_X-ray</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>34.14</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.889</v>
+      </c>
+      <c r="G14" t="n">
+        <v>23.39</v>
+      </c>
+      <c r="H14" t="n">
+        <v>125</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.2324</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>4x4/K64</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>4</v>
+      </c>
+      <c r="C15" t="n">
+        <v>64</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Mammogram</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>36.73</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.9392</v>
+      </c>
+      <c r="G15" t="n">
+        <v>31.56</v>
+      </c>
+      <c r="H15" t="n">
+        <v>98</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.2093</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>4x4/K64</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" t="n">
+        <v>64</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Lung_CT</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.8666</v>
+      </c>
+      <c r="G16" t="n">
+        <v>24.63</v>
+      </c>
+      <c r="H16" t="n">
+        <v>197</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0.2895</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>4x4/K64</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C17" t="n">
+        <v>64</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Brain_MRI</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.9474</v>
+      </c>
+      <c r="G17" t="n">
+        <v>33.49</v>
+      </c>
+      <c r="H17" t="n">
+        <v>142</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0.2446</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>8x8/K64</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>8</v>
+      </c>
+      <c r="C18" t="n">
+        <v>64</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Lena</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>27</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.7517</v>
+      </c>
+      <c r="G18" t="n">
+        <v>35.97</v>
+      </c>
+      <c r="H18" t="n">
+        <v>103</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0.1572</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>8x8/K64</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>8</v>
+      </c>
+      <c r="C19" t="n">
+        <v>64</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Boat</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>26.41</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.7529</v>
+      </c>
+      <c r="G19" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="H19" t="n">
+        <v>107</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0.1674</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>8x8/K64</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>8</v>
+      </c>
+      <c r="C20" t="n">
+        <v>64</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Cameraman</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>26.58</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.8092</v>
+      </c>
+      <c r="G20" t="n">
+        <v>40.22</v>
+      </c>
+      <c r="H20" t="n">
+        <v>98</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0.1485</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>8x8/K64</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>8</v>
+      </c>
+      <c r="C21" t="n">
+        <v>64</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Peppers</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>26.88</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.7027</v>
+      </c>
+      <c r="G21" t="n">
+        <v>36.83</v>
+      </c>
+      <c r="H21" t="n">
+        <v>92</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0.1923</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>8x8/K64</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>8</v>
+      </c>
+      <c r="C22" t="n">
+        <v>64</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Chest_X-ray</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>30.78</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.8033</v>
+      </c>
+      <c r="G22" t="n">
+        <v>35.82</v>
+      </c>
+      <c r="H22" t="n">
+        <v>112</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0.2071</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>8x8/K64</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>8</v>
+      </c>
+      <c r="C23" t="n">
+        <v>64</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Mammogram</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>33.37</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.8854</v>
+      </c>
+      <c r="G23" t="n">
+        <v>40.08</v>
+      </c>
+      <c r="H23" t="n">
+        <v>98</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0.1848</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>8x8/K64</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>8</v>
+      </c>
+      <c r="C24" t="n">
+        <v>64</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Lung_CT</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.738</v>
+      </c>
+      <c r="G24" t="n">
+        <v>37.67</v>
+      </c>
+      <c r="H24" t="n">
+        <v>108</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0.1437</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>8x8/K64</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>8</v>
+      </c>
+      <c r="C25" t="n">
+        <v>64</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Brain_MRI</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>30.03</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.8822</v>
+      </c>
+      <c r="G25" t="n">
+        <v>41.54</v>
+      </c>
+      <c r="H25" t="n">
+        <v>98</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0.1354</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>4x4/K32</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>4</v>
+      </c>
+      <c r="C26" t="n">
+        <v>32</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Lena</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>29.35</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.8186</v>
+      </c>
+      <c r="G26" t="n">
+        <v>30.45</v>
+      </c>
+      <c r="H26" t="n">
+        <v>119</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0.1166</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>4x4/K32</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>4</v>
+      </c>
+      <c r="C27" t="n">
+        <v>32</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Boat</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>28.67</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.8246</v>
+      </c>
+      <c r="G27" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="H27" t="n">
+        <v>117</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0.1096</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>4x4/K32</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>4</v>
+      </c>
+      <c r="C28" t="n">
+        <v>32</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Cameraman</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>29.17</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.876</v>
+      </c>
+      <c r="G28" t="n">
+        <v>39.94</v>
+      </c>
+      <c r="H28" t="n">
+        <v>126</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0.1327</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>4x4/K32</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>4</v>
+      </c>
+      <c r="C29" t="n">
+        <v>32</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Peppers</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>29.23</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0.7653</v>
+      </c>
+      <c r="G29" t="n">
+        <v>32.89</v>
+      </c>
+      <c r="H29" t="n">
+        <v>81</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0.09669999999999999</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>4x4/K32</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>4</v>
+      </c>
+      <c r="C30" t="n">
+        <v>32</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Chest_X-ray</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>32.75</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.8626</v>
+      </c>
+      <c r="G30" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="H30" t="n">
+        <v>92</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0.1138</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>4x4/K32</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>4</v>
+      </c>
+      <c r="C31" t="n">
+        <v>32</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Mammogram</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>35.16</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0.9183</v>
+      </c>
+      <c r="G31" t="n">
+        <v>45.77</v>
+      </c>
+      <c r="H31" t="n">
+        <v>56</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0.0564</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>4x4/K32</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C32" t="n">
+        <v>32</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Lung_CT</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>27.53</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.8278</v>
+      </c>
+      <c r="G32" t="n">
+        <v>34.68</v>
+      </c>
+      <c r="H32" t="n">
+        <v>161</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0.1619</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>4x4/K32</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>4</v>
+      </c>
+      <c r="C33" t="n">
+        <v>32</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Brain_MRI</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>33.02</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0.9284</v>
+      </c>
+      <c r="G33" t="n">
+        <v>43.79</v>
+      </c>
+      <c r="H33" t="n">
+        <v>103</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0.1046</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>4x4/K128</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>4</v>
+      </c>
+      <c r="C34" t="n">
+        <v>128</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Lena</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>31.44</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.8652</v>
+      </c>
+      <c r="G34" t="n">
+        <v>17.92</v>
+      </c>
+      <c r="H34" t="n">
+        <v>210</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0.6252</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>4x4/K128</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>4</v>
+      </c>
+      <c r="C35" t="n">
+        <v>128</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Boat</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>30.62</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0.8743</v>
+      </c>
+      <c r="G35" t="n">
+        <v>19.72</v>
+      </c>
+      <c r="H35" t="n">
+        <v>191</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0.519</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>4x4/K128</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>4</v>
+      </c>
+      <c r="C36" t="n">
+        <v>128</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Cameraman</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0.9232</v>
+      </c>
+      <c r="G36" t="n">
+        <v>21.29</v>
+      </c>
+      <c r="H36" t="n">
+        <v>203</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0.5809</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>4x4/K128</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>4</v>
+      </c>
+      <c r="C37" t="n">
+        <v>128</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Peppers</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>31.05</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0.8068</v>
+      </c>
+      <c r="G37" t="n">
+        <v>18.63</v>
+      </c>
+      <c r="H37" t="n">
+        <v>168</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0.5386</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>4x4/K128</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>4</v>
+      </c>
+      <c r="C38" t="n">
+        <v>128</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Chest_X-ray</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>35.43</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0.9089</v>
+      </c>
+      <c r="G38" t="n">
+        <v>17.61</v>
+      </c>
+      <c r="H38" t="n">
+        <v>177</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0.6054</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>4x4/K128</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>4</v>
+      </c>
+      <c r="C39" t="n">
+        <v>128</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Mammogram</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>38.59</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0.953</v>
+      </c>
+      <c r="G39" t="n">
+        <v>22.24</v>
+      </c>
+      <c r="H39" t="n">
+        <v>132</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0.4529</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>4x4/K128</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>4</v>
+      </c>
+      <c r="C40" t="n">
+        <v>128</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Lung_CT</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>30.13</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0.8925999999999999</v>
+      </c>
+      <c r="G40" t="n">
+        <v>18.55</v>
+      </c>
+      <c r="H40" t="n">
+        <v>224</v>
+      </c>
+      <c r="I40" t="n">
+        <v>0.4837</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>4x4/K128</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>4</v>
+      </c>
+      <c r="C41" t="n">
+        <v>128</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Brain_MRI</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>35.73</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0.9588</v>
+      </c>
+      <c r="G41" t="n">
+        <v>25.13</v>
+      </c>
+      <c r="H41" t="n">
+        <v>168</v>
+      </c>
+      <c r="I41" t="n">
+        <v>0.4413</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>method</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>setting</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>PSNR_dB</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>SSIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Lena</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>4x4 K=64</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="E2" t="n">
+        <v>30.44</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.8431</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Lena</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>JPEG</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>quality=21</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>23.37</v>
+      </c>
+      <c r="E3" t="n">
+        <v>33.14</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.8767</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Lena</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>JPEG 2000</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>target CR=23.50</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>23.53</v>
+      </c>
+      <c r="E4" t="n">
+        <v>35.48</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.9059</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Boat</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>4x4 K=64</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>26.54</v>
+      </c>
+      <c r="E5" t="n">
+        <v>29.65</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.8522</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Boat</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>JPEG</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>quality=17</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>26.41</v>
+      </c>
+      <c r="E6" t="n">
+        <v>31.37</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.8705000000000001</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Boat</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>JPEG 2000</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>target CR=26.54</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>26.53</v>
+      </c>
+      <c r="E7" t="n">
+        <v>33.64</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.9051</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Cameraman</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>4x4 K=64</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>28.88</v>
+      </c>
+      <c r="E8" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.9031</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Cameraman</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>JPEG</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>quality=17</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>29.23</v>
+      </c>
+      <c r="E9" t="n">
+        <v>34.01</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.9173</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Cameraman</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>JPEG 2000</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>target CR=28.88</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>28.85</v>
+      </c>
+      <c r="E10" t="n">
+        <v>37.17</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.9446</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Peppers</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>4x4 K=64</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>24.75</v>
+      </c>
+      <c r="E11" t="n">
+        <v>30.24</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.7875</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Peppers</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>JPEG</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>quality=21</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>24.92</v>
+      </c>
+      <c r="E12" t="n">
+        <v>32.24</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.8103</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Peppers</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>JPEG 2000</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>target CR=24.75</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>24.83</v>
+      </c>
+      <c r="E13" t="n">
+        <v>33.42</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.831</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Chest_X-ray</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>4x4 K=64</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>23.39</v>
+      </c>
+      <c r="E14" t="n">
+        <v>34.14</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.889</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Chest_X-ray</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>JPEG</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>quality=28</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>22.82</v>
+      </c>
+      <c r="E15" t="n">
+        <v>36.88</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.919</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Chest_X-ray</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>JPEG 2000</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>target CR=23.39</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>23.64</v>
+      </c>
+      <c r="E16" t="n">
+        <v>39.4</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.947</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Mammogram</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>4x4 K=64</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>31.56</v>
+      </c>
+      <c r="E17" t="n">
+        <v>36.73</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.9392</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Mammogram</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>JPEG</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>quality=36</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>31.47</v>
+      </c>
+      <c r="E18" t="n">
+        <v>40.94</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.9540999999999999</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Mammogram</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>JPEG 2000</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>target CR=31.56</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>32.59</v>
+      </c>
+      <c r="E19" t="n">
+        <v>43.58</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.9717</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Lung_CT</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>4x4 K=64</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>24.63</v>
+      </c>
+      <c r="E20" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.8666</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Lung_CT</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>JPEG</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>quality=13</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>24.52</v>
+      </c>
+      <c r="E21" t="n">
+        <v>31.22</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.8743</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Lung_CT</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>JPEG 2000</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>target CR=24.63</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>25.06</v>
+      </c>
+      <c r="E22" t="n">
+        <v>33.13</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.9016999999999999</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Brain_MRI</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>4x4 K=64</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>33.49</v>
+      </c>
+      <c r="E23" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.9474</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Brain_MRI</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>JPEG</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>quality=25</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>33.39</v>
+      </c>
+      <c r="E24" t="n">
+        <v>38.66</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.9175</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Brain_MRI</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>JPEG 2000</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>target CR=33.49</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>33.44</v>
+      </c>
+      <c r="E25" t="n">
+        <v>42.11</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.9756</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>CR_fixed8</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>CR_fixed6</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>CR_delta_huffman</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>gain_over_6bit_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Lena</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>15.06</v>
+      </c>
+      <c r="C2" t="n">
+        <v>19.69</v>
+      </c>
+      <c r="D2" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="E2" t="n">
+        <v>19.3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Boat</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>15.06</v>
+      </c>
+      <c r="C3" t="n">
+        <v>19.69</v>
+      </c>
+      <c r="D3" t="n">
+        <v>26.54</v>
+      </c>
+      <c r="E3" t="n">
+        <v>34.8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Cameraman</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>15.06</v>
+      </c>
+      <c r="C4" t="n">
+        <v>19.69</v>
+      </c>
+      <c r="D4" t="n">
+        <v>28.88</v>
+      </c>
+      <c r="E4" t="n">
+        <v>46.7</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Peppers</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>15.06</v>
+      </c>
+      <c r="C5" t="n">
+        <v>19.69</v>
+      </c>
+      <c r="D5" t="n">
+        <v>24.75</v>
+      </c>
+      <c r="E5" t="n">
+        <v>25.7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Chest X-ray</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>15.06</v>
+      </c>
+      <c r="C6" t="n">
+        <v>19.69</v>
+      </c>
+      <c r="D6" t="n">
+        <v>23.39</v>
+      </c>
+      <c r="E6" t="n">
+        <v>18.8</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Mammogram</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>15.06</v>
+      </c>
+      <c r="C7" t="n">
+        <v>19.69</v>
+      </c>
+      <c r="D7" t="n">
+        <v>31.56</v>
+      </c>
+      <c r="E7" t="n">
+        <v>60.3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Lung CT</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>15.06</v>
+      </c>
+      <c r="C8" t="n">
+        <v>19.69</v>
+      </c>
+      <c r="D8" t="n">
+        <v>24.63</v>
+      </c>
+      <c r="E8" t="n">
+        <v>25.1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Brain MRI</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>15.06</v>
+      </c>
+      <c r="C9" t="n">
+        <v>19.69</v>
+      </c>
+      <c r="D9" t="n">
+        <v>33.49</v>
+      </c>
+      <c r="E9" t="n">
+        <v>70.09999999999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>